<commit_message>
QLDA: Import DeXuatChuyenTiep — thêm cột Dự án và query duAnId trên API tải mẫu
Cho phép import ngoài dự án bằng cách chọn dự án từng dòng trong Excel.
Template bỏ STT, thêm dropdown $cbo1; API template lọc DTH hoặc theo duAnId.
Handler resolve TenDuAn và BuocHienTaiId khi không gửi duAnId/buocId form.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/QLDA.WebApi/PrintTemplates/Import_DeXuatChuTruongChuyenTiep.xlsx
+++ b/QLDA.WebApi/PrintTemplates/Import_DeXuatChuTruongChuyenTiep.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SER\QLDA.WebApi\PrintTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE89A32-63EE-4C12-8F08-CF5D4EA31D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F975A720-6C94-4DD0-8BEC-C05F5ADB4F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,16 +17,25 @@
     <sheet name="Danh mục" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+  <si>
+    <t>ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
+TRUNG TÂM CHUYỂN ĐỔI SỐ</t>
+  </si>
+  <si>
+    <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
+Độc lập - Tự do - Hạnh phúc</t>
+  </si>
   <si>
     <t>MẪU IMPORT ĐỀ XUẤT CHỦ TRƯƠNG CHUYỂN TIẾP</t>
   </si>
   <si>
-    <t>STT</t>
+    <t>Dự án</t>
   </si>
   <si>
     <t>Số liệu giải ngân</t>
@@ -44,7 +53,7 @@
     <t>Khối lượng dự kiến hoàn thành</t>
   </si>
   <si>
-    <t>1, 2, 3...</t>
+    <t>$cbo1</t>
   </si>
   <si>
     <t>Nhập số tiền (đồng)</t>
@@ -53,46 +62,13 @@
     <t>Mô tả khối lượng</t>
   </si>
   <si>
-    <t>Dự án</t>
-  </si>
-  <si>
     <t>Bước</t>
   </si>
   <si>
-    <t>$cbo1</t>
-  </si>
-  <si>
     <t>$cbo2</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">ỦY BAN NHÂN DÂN THÀNH PHỐ HỒ CHÍ MINH
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>TRUNG TÂM CHUYỂN ĐỔI SỐ</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>Độc lập - Tự do - Hạnh phúc</t>
-    </r>
+    <t>Chọn từ danh sách</t>
   </si>
 </sst>
 </file>
@@ -132,16 +108,16 @@
       <family val="1"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -189,26 +165,32 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -219,11 +201,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -231,11 +211,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -243,11 +221,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -255,11 +231,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -267,11 +241,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -279,11 +251,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -291,11 +261,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -303,11 +271,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -315,11 +281,9 @@
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
-        <u val="none"/>
         <vertAlign val="baseline"/>
         <name val="Times New Roman"/>
         <family val="1"/>
-        <scheme val="none"/>
       </font>
     </dxf>
   </dxfs>
@@ -336,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DeXuatChuyenTiepImport" displayName="DeXuatChuyenTiepImport" ref="A5:F7" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DeXuatChuyenTiepImport" displayName="DeXuatChuyenTiepImport" ref="A5:F7" headerRowDxfId="8" dataDxfId="7" totalsRowDxfId="6">
   <autoFilter ref="A5:F7" xr:uid="{00000000-0009-0000-0100-000001000000}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -346,12 +310,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="STT" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Số liệu giải ngân" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Ước giải ngân" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Nhu cầu kinh phí" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Khối lượng đã hoàn thành" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Khối lượng dự kiến hoàn thành" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="STT" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Số liệu giải ngân" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Ước giải ngân" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Nhu cầu kinh phí" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Khối lượng đã hoàn thành" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Khối lượng dự kiến hoàn thành" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -665,204 +629,207 @@
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" style="6" customWidth="1"/>
-    <col min="2" max="2" width="28.21875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="24.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="40.77734375" style="6" customWidth="1"/>
-    <col min="6" max="6" width="37.88671875" style="6" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="47.33203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="28.21875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="23.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="24.33203125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="40.77734375" style="3" customWidth="1"/>
+    <col min="6" max="6" width="37.88671875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="9"/>
+    </row>
+    <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="5"/>
-    </row>
-    <row r="2" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-    </row>
-    <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-    </row>
-    <row r="5" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -870,6 +837,7 @@
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="E1:F2"/>
   </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -884,15 +852,15 @@
   <sheetData>
     <row r="3" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>

</xml_diff>